<commit_message>
Complete team list: add Vivek LinkedIn + Shreyash location (Nashik)
</commit_message>
<xml_diff>
--- a/IDEAS_team_members.xlsx
+++ b/IDEAS_team_members.xlsx
@@ -184,7 +184,11 @@
           <t xml:space="preserve">25B2269</t>
         </is>
       </c>
-      <c r="J3"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.linkedin.com/in/vivek-gupta-283912388</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">Male</t>
@@ -222,7 +226,11 @@
           <t xml:space="preserve">B.Tech</t>
         </is>
       </c>
-      <c r="F4"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nashik, Maharashtra</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t xml:space="preserve">Mechanical Engineering</t>

</xml_diff>